<commit_message>
Update ID spreadsheet (x2)
</commit_message>
<xml_diff>
--- a/GHtoRB2_songids.xlsx
+++ b/GHtoRB2_songids.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\RBDLC\reference\!GHtoRB2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54C16938-AF3D-4009-A640-209F5292BEBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94DD2A12-D48E-4E86-B9C3-CBF6185B7A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{AE99FE45-D305-4219-A47C-654285C6D506}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1408" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1472" uniqueCount="324">
   <si>
     <t>Last Updated: 3/13/26</t>
   </si>
@@ -11089,7 +11089,9 @@
       <c r="D704" s="3">
         <v>4200699</v>
       </c>
-      <c r="E704" s="3"/>
+      <c r="E704" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F704" s="3"/>
       <c r="G704" s="3"/>
     </row>
@@ -11106,7 +11108,9 @@
       <c r="D705" s="3">
         <v>4200700</v>
       </c>
-      <c r="E705" s="3"/>
+      <c r="E705" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F705" s="3"/>
       <c r="G705" s="3"/>
     </row>
@@ -11123,7 +11127,9 @@
       <c r="D706" s="3">
         <v>4200701</v>
       </c>
-      <c r="E706" s="3"/>
+      <c r="E706" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F706" s="3"/>
       <c r="G706" s="3"/>
     </row>
@@ -11140,7 +11146,9 @@
       <c r="D707" s="3">
         <v>4200702</v>
       </c>
-      <c r="E707" s="3"/>
+      <c r="E707" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F707" s="3"/>
       <c r="G707" s="3"/>
     </row>
@@ -11157,7 +11165,9 @@
       <c r="D708" s="3">
         <v>4200703</v>
       </c>
-      <c r="E708" s="3"/>
+      <c r="E708" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F708" s="3"/>
       <c r="G708" s="3"/>
     </row>
@@ -11174,7 +11184,9 @@
       <c r="D709" s="3">
         <v>4200704</v>
       </c>
-      <c r="E709" s="3"/>
+      <c r="E709" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F709" s="3"/>
       <c r="G709" s="3"/>
     </row>
@@ -11191,7 +11203,9 @@
       <c r="D710" s="3">
         <v>4200705</v>
       </c>
-      <c r="E710" s="3"/>
+      <c r="E710" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F710" s="3"/>
       <c r="G710" s="3"/>
     </row>
@@ -11208,7 +11222,9 @@
       <c r="D711" s="3">
         <v>4200706</v>
       </c>
-      <c r="E711" s="3"/>
+      <c r="E711" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F711" s="3"/>
       <c r="G711" s="3"/>
     </row>
@@ -11225,7 +11241,9 @@
       <c r="D712" s="3">
         <v>4200707</v>
       </c>
-      <c r="E712" s="3"/>
+      <c r="E712" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F712" s="3"/>
       <c r="G712" s="3"/>
     </row>
@@ -11242,7 +11260,9 @@
       <c r="D713" s="3">
         <v>4200708</v>
       </c>
-      <c r="E713" s="3"/>
+      <c r="E713" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F713" s="3"/>
       <c r="G713" s="3"/>
     </row>
@@ -11259,7 +11279,9 @@
       <c r="D714" s="3">
         <v>4200709</v>
       </c>
-      <c r="E714" s="3"/>
+      <c r="E714" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F714" s="3"/>
       <c r="G714" s="3"/>
     </row>
@@ -11276,7 +11298,9 @@
       <c r="D715" s="3">
         <v>4200710</v>
       </c>
-      <c r="E715" s="3"/>
+      <c r="E715" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F715" s="3"/>
       <c r="G715" s="3"/>
     </row>
@@ -11293,7 +11317,9 @@
       <c r="D716" s="3">
         <v>4200711</v>
       </c>
-      <c r="E716" s="3"/>
+      <c r="E716" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F716" s="3"/>
       <c r="G716" s="3"/>
     </row>
@@ -11310,7 +11336,9 @@
       <c r="D717" s="3">
         <v>4200712</v>
       </c>
-      <c r="E717" s="3"/>
+      <c r="E717" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F717" s="3"/>
       <c r="G717" s="3"/>
     </row>
@@ -11327,7 +11355,9 @@
       <c r="D718" s="3">
         <v>4200713</v>
       </c>
-      <c r="E718" s="3"/>
+      <c r="E718" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F718" s="3"/>
       <c r="G718" s="3"/>
     </row>
@@ -11344,7 +11374,9 @@
       <c r="D719" s="3">
         <v>4200714</v>
       </c>
-      <c r="E719" s="3"/>
+      <c r="E719" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F719" s="3"/>
       <c r="G719" s="3"/>
     </row>
@@ -11361,7 +11393,9 @@
       <c r="D720" s="3">
         <v>4200715</v>
       </c>
-      <c r="E720" s="3"/>
+      <c r="E720" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F720" s="3"/>
       <c r="G720" s="3"/>
     </row>
@@ -11378,7 +11412,9 @@
       <c r="D721" s="3">
         <v>4200716</v>
       </c>
-      <c r="E721" s="3"/>
+      <c r="E721" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F721" s="3"/>
       <c r="G721" s="3"/>
     </row>
@@ -11395,7 +11431,9 @@
       <c r="D722" s="3">
         <v>4200717</v>
       </c>
-      <c r="E722" s="3"/>
+      <c r="E722" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F722" s="3"/>
       <c r="G722" s="3"/>
     </row>
@@ -11412,7 +11450,9 @@
       <c r="D723" s="3">
         <v>4200718</v>
       </c>
-      <c r="E723" s="3"/>
+      <c r="E723" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F723" s="3"/>
       <c r="G723" s="3"/>
     </row>
@@ -11429,7 +11469,9 @@
       <c r="D724" s="3">
         <v>4200719</v>
       </c>
-      <c r="E724" s="3"/>
+      <c r="E724" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F724" s="3"/>
       <c r="G724" s="3"/>
     </row>
@@ -11446,7 +11488,9 @@
       <c r="D725" s="3">
         <v>4200720</v>
       </c>
-      <c r="E725" s="3"/>
+      <c r="E725" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F725" s="3"/>
       <c r="G725" s="3"/>
     </row>
@@ -11528,7 +11572,9 @@
       <c r="D731" s="3">
         <v>4200726</v>
       </c>
-      <c r="E731" s="3"/>
+      <c r="E731" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F731" s="3"/>
       <c r="G731" s="3"/>
     </row>
@@ -11649,7 +11695,9 @@
       <c r="D740" s="3">
         <v>4200735</v>
       </c>
-      <c r="E740" s="3"/>
+      <c r="E740" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F740" s="3"/>
       <c r="G740" s="3"/>
     </row>
@@ -11783,7 +11831,9 @@
       <c r="D750" s="3">
         <v>4200745</v>
       </c>
-      <c r="E750" s="3"/>
+      <c r="E750" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F750" s="3"/>
       <c r="G750" s="3"/>
     </row>
@@ -11878,7 +11928,9 @@
       <c r="D757" s="3">
         <v>4200752</v>
       </c>
-      <c r="E757" s="3"/>
+      <c r="E757" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F757" s="3"/>
       <c r="G757" s="3"/>
     </row>
@@ -12025,7 +12077,9 @@
       <c r="D768" s="3">
         <v>4200763</v>
       </c>
-      <c r="E768" s="3"/>
+      <c r="E768" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F768" s="3"/>
       <c r="G768" s="3"/>
     </row>
@@ -12042,7 +12096,9 @@
       <c r="D769" s="3">
         <v>4200764</v>
       </c>
-      <c r="E769" s="3"/>
+      <c r="E769" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F769" s="3"/>
       <c r="G769" s="3"/>
     </row>
@@ -12059,7 +12115,9 @@
       <c r="D770" s="3">
         <v>4200765</v>
       </c>
-      <c r="E770" s="3"/>
+      <c r="E770" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F770" s="3"/>
       <c r="G770" s="3"/>
     </row>
@@ -12076,7 +12134,9 @@
       <c r="D771" s="3">
         <v>4200766</v>
       </c>
-      <c r="E771" s="3"/>
+      <c r="E771" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F771" s="3"/>
       <c r="G771" s="3"/>
     </row>
@@ -12093,7 +12153,9 @@
       <c r="D772" s="3">
         <v>4200767</v>
       </c>
-      <c r="E772" s="3"/>
+      <c r="E772" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F772" s="3"/>
       <c r="G772" s="3"/>
     </row>
@@ -12110,7 +12172,9 @@
       <c r="D773" s="3">
         <v>4200768</v>
       </c>
-      <c r="E773" s="3"/>
+      <c r="E773" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F773" s="3"/>
       <c r="G773" s="3"/>
     </row>
@@ -12127,7 +12191,9 @@
       <c r="D774" s="3">
         <v>4200769</v>
       </c>
-      <c r="E774" s="3"/>
+      <c r="E774" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F774" s="3"/>
       <c r="G774" s="3"/>
     </row>
@@ -12144,7 +12210,9 @@
       <c r="D775" s="3">
         <v>4200770</v>
       </c>
-      <c r="E775" s="3"/>
+      <c r="E775" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F775" s="3"/>
       <c r="G775" s="3"/>
     </row>
@@ -12161,7 +12229,9 @@
       <c r="D776" s="3">
         <v>4200771</v>
       </c>
-      <c r="E776" s="3"/>
+      <c r="E776" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F776" s="3"/>
       <c r="G776" s="3"/>
     </row>
@@ -12178,7 +12248,9 @@
       <c r="D777" s="3">
         <v>4200772</v>
       </c>
-      <c r="E777" s="3"/>
+      <c r="E777" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F777" s="3"/>
       <c r="G777" s="3"/>
     </row>
@@ -12195,7 +12267,9 @@
       <c r="D778" s="3">
         <v>4200773</v>
       </c>
-      <c r="E778" s="3"/>
+      <c r="E778" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F778" s="3"/>
       <c r="G778" s="3"/>
     </row>
@@ -12212,7 +12286,9 @@
       <c r="D779" s="3">
         <v>4200774</v>
       </c>
-      <c r="E779" s="3"/>
+      <c r="E779" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F779" s="3"/>
       <c r="G779" s="3"/>
     </row>
@@ -12229,7 +12305,9 @@
       <c r="D780" s="3">
         <v>4200775</v>
       </c>
-      <c r="E780" s="3"/>
+      <c r="E780" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F780" s="3"/>
       <c r="G780" s="3"/>
     </row>
@@ -12246,7 +12324,9 @@
       <c r="D781" s="3">
         <v>4200776</v>
       </c>
-      <c r="E781" s="3"/>
+      <c r="E781" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F781" s="3"/>
       <c r="G781" s="3"/>
     </row>
@@ -12263,7 +12343,9 @@
       <c r="D782" s="3">
         <v>4200777</v>
       </c>
-      <c r="E782" s="3"/>
+      <c r="E782" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F782" s="3"/>
       <c r="G782" s="3"/>
     </row>
@@ -12280,7 +12362,9 @@
       <c r="D783" s="3">
         <v>4200778</v>
       </c>
-      <c r="E783" s="3"/>
+      <c r="E783" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F783" s="3"/>
       <c r="G783" s="3"/>
     </row>
@@ -12297,7 +12381,9 @@
       <c r="D784" s="3">
         <v>4200779</v>
       </c>
-      <c r="E784" s="3"/>
+      <c r="E784" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F784" s="3"/>
       <c r="G784" s="3"/>
     </row>
@@ -12314,7 +12400,9 @@
       <c r="D785" s="3">
         <v>4200780</v>
       </c>
-      <c r="E785" s="3"/>
+      <c r="E785" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F785" s="3"/>
       <c r="G785" s="3"/>
     </row>
@@ -12331,7 +12419,9 @@
       <c r="D786" s="3">
         <v>4200781</v>
       </c>
-      <c r="E786" s="3"/>
+      <c r="E786" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F786" s="3"/>
       <c r="G786" s="3"/>
     </row>
@@ -12348,7 +12438,9 @@
       <c r="D787" s="3">
         <v>4200782</v>
       </c>
-      <c r="E787" s="3"/>
+      <c r="E787" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F787" s="3"/>
       <c r="G787" s="3"/>
     </row>
@@ -12365,7 +12457,9 @@
       <c r="D788" s="3">
         <v>4200783</v>
       </c>
-      <c r="E788" s="3"/>
+      <c r="E788" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F788" s="3"/>
       <c r="G788" s="3"/>
     </row>
@@ -12382,7 +12476,9 @@
       <c r="D789" s="3">
         <v>4200784</v>
       </c>
-      <c r="E789" s="3"/>
+      <c r="E789" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F789" s="3"/>
       <c r="G789" s="3"/>
     </row>
@@ -12399,7 +12495,9 @@
       <c r="D790" s="3">
         <v>4200785</v>
       </c>
-      <c r="E790" s="3"/>
+      <c r="E790" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F790" s="3"/>
       <c r="G790" s="3"/>
     </row>
@@ -12416,7 +12514,9 @@
       <c r="D791" s="3">
         <v>4200786</v>
       </c>
-      <c r="E791" s="3"/>
+      <c r="E791" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F791" s="3"/>
       <c r="G791" s="3"/>
     </row>
@@ -12433,7 +12533,9 @@
       <c r="D792" s="3">
         <v>4200787</v>
       </c>
-      <c r="E792" s="3"/>
+      <c r="E792" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F792" s="3"/>
       <c r="G792" s="3"/>
     </row>
@@ -12450,7 +12552,9 @@
       <c r="D793" s="3">
         <v>4200788</v>
       </c>
-      <c r="E793" s="3"/>
+      <c r="E793" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F793" s="3"/>
       <c r="G793" s="3"/>
     </row>
@@ -12467,7 +12571,9 @@
       <c r="D794" s="3">
         <v>4200789</v>
       </c>
-      <c r="E794" s="3"/>
+      <c r="E794" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F794" s="3"/>
       <c r="G794" s="3"/>
     </row>
@@ -12484,7 +12590,9 @@
       <c r="D795" s="3">
         <v>4200790</v>
       </c>
-      <c r="E795" s="3"/>
+      <c r="E795" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F795" s="3"/>
       <c r="G795" s="3"/>
     </row>
@@ -12501,7 +12609,9 @@
       <c r="D796" s="3">
         <v>4200791</v>
       </c>
-      <c r="E796" s="3"/>
+      <c r="E796" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F796" s="3"/>
       <c r="G796" s="3"/>
     </row>
@@ -12518,7 +12628,9 @@
       <c r="D797" s="3">
         <v>4200792</v>
       </c>
-      <c r="E797" s="3"/>
+      <c r="E797" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F797" s="3"/>
       <c r="G797" s="3"/>
     </row>
@@ -12535,7 +12647,9 @@
       <c r="D798" s="3">
         <v>4200793</v>
       </c>
-      <c r="E798" s="3"/>
+      <c r="E798" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F798" s="3"/>
       <c r="G798" s="3"/>
     </row>
@@ -12552,7 +12666,9 @@
       <c r="D799" s="3">
         <v>4200794</v>
       </c>
-      <c r="E799" s="3"/>
+      <c r="E799" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F799" s="3"/>
       <c r="G799" s="3"/>
     </row>
@@ -12569,7 +12685,9 @@
       <c r="D800" s="3">
         <v>4200795</v>
       </c>
-      <c r="E800" s="3"/>
+      <c r="E800" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F800" s="3"/>
       <c r="G800" s="3"/>
     </row>
@@ -12586,7 +12704,9 @@
       <c r="D801" s="3">
         <v>4200796</v>
       </c>
-      <c r="E801" s="3"/>
+      <c r="E801" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F801" s="3"/>
       <c r="G801" s="3"/>
     </row>
@@ -12603,7 +12723,9 @@
       <c r="D802" s="3">
         <v>4200797</v>
       </c>
-      <c r="E802" s="3"/>
+      <c r="E802" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F802" s="3"/>
       <c r="G802" s="3"/>
     </row>
@@ -12620,7 +12742,9 @@
       <c r="D803" s="3">
         <v>4200798</v>
       </c>
-      <c r="E803" s="3"/>
+      <c r="E803" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F803" s="3"/>
       <c r="G803" s="3"/>
     </row>
@@ -12637,7 +12761,9 @@
       <c r="D804" s="3">
         <v>4200799</v>
       </c>
-      <c r="E804" s="3"/>
+      <c r="E804" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F804" s="3"/>
       <c r="G804" s="3"/>
     </row>
@@ -12654,7 +12780,9 @@
       <c r="D805" s="3">
         <v>4200800</v>
       </c>
-      <c r="E805" s="3"/>
+      <c r="E805" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="F805" s="3"/>
       <c r="G805" s="3"/>
     </row>

</xml_diff>